<commit_message>
Added FirstOrDefault and Take in Program.cs and Excel Some other minor fixes
</commit_message>
<xml_diff>
--- a/Week12/W12_1/Material/LINQ_Methods.xlsx
+++ b/Week12/W12_1/Material/LINQ_Methods.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hrnl-my.sharepoint.com/personal/heiga_hr_nl/Documents/Documents/GitHub/OODP/Week12/W12_1/Material/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hrnl-my.sharepoint.com/personal/bardr_hr_nl/Documents/2025-2026 SEM2/OODP/Lab 26/Lessons/W12_1 LINQ/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="185" documentId="8_{A73AFA0F-A3BC-4E7C-8F2D-DAC76A5178A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42B45D9F-00DF-4AE2-B451-2A9DFC54366A}"/>
+  <xr:revisionPtr revIDLastSave="225" documentId="8_{A73AFA0F-A3BC-4E7C-8F2D-DAC76A5178A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3A53C69-4389-4EC2-A060-53E28F455D14}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" activeTab="1" xr2:uid="{FF78A85B-DB44-4C66-B539-359ADDCC737D}"/>
+    <workbookView xWindow="-2355" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{FF78A85B-DB44-4C66-B539-359ADDCC737D}"/>
   </bookViews>
   <sheets>
     <sheet name="long" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="129">
   <si>
     <t>Classification</t>
   </si>
@@ -419,6 +419,39 @@
   </si>
   <si>
     <t>int min = numbers.Min();</t>
+  </si>
+  <si>
+    <t>FirstOrDefault</t>
+  </si>
+  <si>
+    <t>Returns the first element of the sequence that satisfies a condition</t>
+  </si>
+  <si>
+    <t>None or a transform function to apply to each element.</t>
+  </si>
+  <si>
+    <t>None or a function to test each element for a condition</t>
+  </si>
+  <si>
+    <t>Take</t>
+  </si>
+  <si>
+    <t>int first = numbers.FirstOrDefault();</t>
+  </si>
+  <si>
+    <t>default(TSource) if source is empty; otherwise, the first element in source.</t>
+  </si>
+  <si>
+    <t>Returns a specified number of contiguous elements from the start of a sequence.</t>
+  </si>
+  <si>
+    <t>The number of elements to return</t>
+  </si>
+  <si>
+    <t>An IEnumerable&lt;T&gt; that contains the specified number of elements from the start of the input sequence.</t>
+  </si>
+  <si>
+    <t>int[] first3 = numbers.Take(3).ToArray();</t>
   </si>
 </sst>
 </file>
@@ -843,10 +876,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -1144,7 +1173,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545EF625-53DA-45DD-92E6-43AFBE5F4585}">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="1" bestFit="1" customWidth="1"/>
@@ -1432,7 +1461,7 @@
         <v>50</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>71</v>
@@ -1450,7 +1479,7 @@
         <v>51</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>73</v>
@@ -1468,7 +1497,7 @@
         <v>84</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>32</v>
+        <v>121</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>85</v>
@@ -1486,7 +1515,7 @@
         <v>52</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>72</v>
@@ -1495,46 +1524,46 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="16" t="s">
         <v>55</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>32</v>
+        <v>121</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="10" t="s">
-        <v>98</v>
+        <v>74</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="17"/>
       <c r="B20" s="5" t="s">
-        <v>23</v>
+        <v>118</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>56</v>
+        <v>119</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>32</v>
+        <v>121</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>74</v>
+        <v>124</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A21" s="18"/>
+      <c r="A21" s="17"/>
       <c r="B21" s="5" t="s">
         <v>22</v>
       </c>
@@ -1542,7 +1571,7 @@
         <v>57</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>32</v>
+        <v>121</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>75</v>
@@ -1551,23 +1580,59 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="17"/>
+      <c r="B22" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="18"/>
+      <c r="B23" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B24" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C24" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F24" s="9" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1577,7 +1642,7 @@
     <mergeCell ref="A15:A18"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="A19:A23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1587,7 +1652,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B5E5DE1-9389-43DF-A9E2-94A89FA9ED77}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.54296875" style="2" bestFit="1" customWidth="1"/>
@@ -1748,31 +1813,39 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B21" s="13" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="42.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+    <row r="22" spans="1:2" ht="42.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B22" s="14" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+    <row r="23" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B23" s="13" t="s">
         <v>101</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C22">
-    <sortCondition ref="C2:C22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C23">
+    <sortCondition ref="C2:C23"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>